<commit_message>
fix(templates): drop stray column-level borders from the blanked templates
The original forms border columns E/H/I at the column level, so once the data
rows were removed those borders kept running down the empty area while the
other columns (whose borders were cell-level on the deleted rows) showed none.
Strip the bordered <col> styles when blanking, so the template is consistent:
a uniformly bordered title + header row, clean empty grid below.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/templates/Staf.xlsx
+++ b/assets/templates/Staf.xlsx
@@ -1437,11 +1437,11 @@
     <col min="2" max="2" width="15.85546875" style="19" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="30.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.85546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="24.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="44.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.85546875" style="7" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.85546875" style="58" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="37.28515625" style="37" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1507,11 +1507,11 @@
     <col min="2" max="2" width="15.85546875" style="19" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="31.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.85546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="24.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="43.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.85546875" style="7" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.85546875" style="34" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9.140625" style="1"/>
   </cols>
   <sheetData>
@@ -1576,11 +1576,11 @@
     <col min="2" max="2" width="16.28515625" style="19" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="30" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.85546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="25.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="43.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.85546875" style="7" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.85546875" style="34" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="16.28515625" style="37" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1646,11 +1646,11 @@
     <col min="2" max="2" width="15.85546875" style="19" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="31.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.85546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="24.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="43.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.85546875" style="7" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.85546875" style="34" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="14.85546875" style="37" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1716,11 +1716,11 @@
     <col min="2" max="2" width="15.85546875" style="19" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="31.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.85546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="24.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="38.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.85546875" style="7" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.85546875" style="34" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="7.42578125" style="37" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1785,11 +1785,11 @@
     <col min="2" max="2" width="15.85546875" style="19" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="31.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.85546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="24.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="38.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.85546875" style="7" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.85546875" style="34" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="7.42578125" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1854,11 +1854,11 @@
     <col min="2" max="2" width="15.85546875" style="19" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="31.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.85546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="24.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="38.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.85546875" style="7" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.85546875" style="34" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="7.42578125" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1923,11 +1923,11 @@
     <col min="2" max="2" width="15.85546875" style="19" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="31.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.85546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="24.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="38.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.85546875" style="7" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.85546875" style="34" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="7.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="11" max="12" width="9.140625" style="31"/>
   </cols>
@@ -1995,11 +1995,11 @@
     <col min="2" max="2" width="15.85546875" style="19" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="31.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.85546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="24.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="38.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.85546875" style="7" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.85546875" style="34" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="16.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="11" max="12" width="9.140625" style="31"/>
   </cols>
@@ -2067,11 +2067,11 @@
     <col min="2" max="2" width="15.85546875" style="19" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="31.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.85546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="24.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="38.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.85546875" style="7" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.85546875" style="34" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="13.28515625" style="31" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="16.140625" style="31" bestFit="1" customWidth="1"/>
   </cols>

</xml_diff>